<commit_message>
chore: switch to dev-only environment and update Registration, Login, docs, scripts and support
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/manual-test-cases/Balances-Wallet-Consistency-EMI-5944/Balances & Wallet Consistency Test_Cases EMI-5944.xlsx
+++ b/docs/manual-test-cases/Balances-Wallet-Consistency-EMI-5944/Balances & Wallet Consistency Test_Cases EMI-5944.xlsx
@@ -20,14 +20,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E Balances Flows" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Consumer Partitioning'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Consumer Idempotency'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lifecycle Ordering Guard'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Consumer Partitioning'!$A$1:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Consumer Idempotency'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lifecycle Ordering Guard'!$A$1:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Statement History Rebuild'!$A$1:$I$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Wallet Balance Recompute'!$A$1:$I$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Bucket Identity Validation'!$A$1:$I$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Stuck Reserve Detection'!$A$1:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Wallet Daily Close'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Wallet Daily Close'!$A$1:$I$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'EMI_MISSING Resolution'!$A$1:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'E2E Balances Flows'!$A$1:$I$21</definedName>
   </definedNames>
@@ -3428,7 +3428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4447,8 +4447,299 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Cutover</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>TC-Partition-21</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>Increasing the Partition Count Does Not Reorder a Wallet In Flight</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" s="28" t="inlineStr">
+        <is>
+          <t>Topic re-keyed on wallet_id and consuming normally; a wallet with postings in flight</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>1. Begin a stream of PENDING/SUCCESS postings for one wallet
+2. Increase the topic partition count while those postings are in flight
+3. Let the stream complete
+4. Read the wallet buckets and compare against a ledger-derived recompute</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>Either the partition change is blocked while events are in flight, or the cutover drains first; in no case are two events for one wallet applied out of commit order. Final buckets match the ledger</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Cutover</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>TC-Partition-22</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>Mixed-Keying Is Actively Detected, Not Only Avoided by Procedure</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E23" s="28" t="inlineStr">
+        <is>
+          <t>A test topic seeded with both entry-id-keyed and wallet_id-keyed events</t>
+        </is>
+      </c>
+      <c r="F23" s="28" t="inlineStr">
+        <is>
+          <t>1. Present the consumer with both keyings on the same topic
+2. Observe consumer behaviour and alerting</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="inlineStr">
+        <is>
+          <t>The consumer detects the mixed keying and refuses to consume, or halts and alerts, rather than silently applying both. The condition is visible in monitoring, not left to the runbook</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I23" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>Keying</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>TC-Partition-23</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>An Event With a Null or Missing wallet_id Is Not Round-Robined</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" s="28" t="inlineStr">
+        <is>
+          <t>Re-keying SMT in place</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>1. Publish a CDC event whose wallet_id is null or absent
+2. Observe the partition it lands on and the consumer outcome</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>The event is routed to a dead-letter path or halts consumption with an alert. It is never given a null key, because a null key round-robins and silently destroys per-wallet ordering</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I24" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Keying</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>TC-Partition-24</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>A Delete or Tombstone Event on an Append-Only Ledger Is Treated as an Anomaly</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E25" s="28" t="inlineStr">
+        <is>
+          <t>Re-keying SMT in place; the ledger is append-only by contract</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>1. Publish a CDC delete/tombstone event for a ledger entry
+2. Observe the consumer</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>The event is rejected and alerted rather than applied. A delete on an append-only ledger indicates upstream corruption and must not silently reduce a balance</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I25" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>TC-Partition-25</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>Commission and VAT Wallet Skew Does Not Create a Hot Partition</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>Production-representative load in which every transaction posts to the shared commission and VAT wallets</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>1. Drive production-volume mixed traffic
+2. Measure per-partition throughput and lag
+3. Identify the partitions owning the commission and VAT wallets</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>Per-partition lag stays inside its alert threshold. Because keying on wallet_id pins these high-traffic wallets to single partitions, the sizing review accounts for the skew rather than assuming even distribution</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>Performance / NFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>Ordering</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>TC-Partition-26</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>Thread-Hashed Processing Keeps One Wallet on One Thread</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>Consumer configured to hash work to threads by wallet_id rather than one thread per partition</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>1. Send interleaved postings for several wallets sharing a partition
+2. Trace which thread handles each wallet</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>A wallet's events are always handled by the same thread and never processed concurrently. Serial application is a property of the wallet, not merely of the partition</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I27" s="29" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I27"/>
   <conditionalFormatting sqref="H2:H21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Passed"</formula>
@@ -4484,7 +4775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5505,8 +5796,251 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>TC-Idem-21</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>The Uniqueness Key Is the Ledger Entry, Not the Transaction</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" s="28" t="inlineStr">
+        <is>
+          <t>Uniqueness constraint in place; a transaction with PENDING and SUCCESS postings</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>1. Deliver the PENDING posting for transaction T
+2. Deliver the SUCCESS posting for the same transaction T
+3. Inspect the projection rows and the buckets</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>Both postings are applied and both projection rows exist. They share a transaction_id but are distinct ledger entries, so the constraint must not reject the second. Keying uniqueness on transaction_id would suppress every lifecycle transition</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>TC-Idem-22</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>A MySQL Binlog Position Compares File First, Then Offset</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E23" s="28" t="inlineStr">
+        <is>
+          <t>Deployment using the MySQL connector, where last_applied_position is binlog file plus position</t>
+        </is>
+      </c>
+      <c r="F23" s="28" t="inlineStr">
+        <is>
+          <t>1. Record a position in file mysql-bin.000009 at a high offset
+2. Deliver an event from file mysql-bin.000010 at a lower offset
+3. Observe whether it is applied</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="inlineStr">
+        <is>
+          <t>The newer event is applied. Comparison orders by file first and offset second; a plain lexicographic or numeric compare on the offset alone would wrongly discard it after a binlog rollover</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I23" s="29" t="inlineStr">
+        <is>
+          <t>Edge / Boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>TC-Idem-23</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>Re-Creating the Connector Does Not Make Old Positions Look Newer</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" s="28" t="inlineStr">
+        <is>
+          <t>A wallet carrying a last_applied_position from the current connector</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>1. Drop and re-create the Debezium connector, forcing a new snapshot
+2. Let it re-emit events
+3. Observe the comparison against stored positions</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>Positions from the new connector are not naively compared against the old ones. Either the position carries a connector generation, or replayed events are recognised as duplicates by entry identity. Balances do not move</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I24" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Concurrency</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>TC-Idem-24</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>The Same Entry Delivered to Two Consumers at Once Has One Effect</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E25" s="28" t="inlineStr">
+        <is>
+          <t>Two consumer instances running; ability to deliver the same entry to both simultaneously</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>1. Deliver one ledger entry to two consumer instances at the same instant
+2. Inspect the projection rows and the wallet buckets</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>Exactly one projection row and one balance effect result. The loser is rejected by the constraint and discarded, not retried into a second application</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I25" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>TC-Idem-25</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>A Discarded Event Is Logged With Its Identity, Not Only Counted</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>Discarded-event metric in place</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>1. Cause a stale and a duplicate event to be discarded
+2. Inspect the log record for each</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>Each discard is recorded with the ledger entry identity, wallet, position and the reason. A counter alone cannot answer which event was dropped, which is what "never dropped without record" requires</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I26"/>
   <conditionalFormatting sqref="H2:H21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Passed"</formula>
@@ -5542,7 +6076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6755,8 +7289,156 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>TC-Lifecycle-25</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>A Redelivered PENDING Does Not Satisfy the Guard Twice</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>Idempotency and the ordering guard both active</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>1. Deliver PENDING for transaction T
+2. Redeliver the identical PENDING
+3. Deliver two SUCCESS postings for T</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>The duplicate PENDING is discarded and does not register a second satisfied predecessor. Only the legitimate SUCCESS applies; the second is handled as a duplicate. Buckets reflect one reservation and one settlement</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>TC-Lifecycle-26</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>A Park Storm Does Not Stall the Consumer</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>Ability to withhold a large number of predecessor postings</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>1. Withhold the PENDING postings for a large batch of transactions
+2. Deliver their SUCCESS postings, forcing mass parking
+3. Observe consumer throughput and the parked store
+4. Release the predecessors</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>The parked store is bounded and does not exhaust memory or disk; unrelated wallets continue to be processed at normal throughput; on release everything converges to correct buckets</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I27" s="29" t="inlineStr">
+        <is>
+          <t>Performance / NFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>TC-Lifecycle-27</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr">
+        <is>
+          <t>Guard State Survives a Consumer Restart</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>Transactions with postings parked awaiting a predecessor</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>1. Park several postings
+2. Restart the consumer
+3. Deliver the missing predecessors</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="inlineStr">
+        <is>
+          <t>Parked postings and the per-transaction applied stage survive the restart and resolve normally. Guard state is durable, not held only in memory, or the restart would silently apply postings out of order</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I28" s="29" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I25"/>
+  <autoFilter ref="A1:I28"/>
   <conditionalFormatting sqref="H2:H25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Passed"</formula>
@@ -13531,7 +14213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -14547,8 +15229,444 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-21</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>Only the Finance Lead May Sign Off a Variance Day</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" s="28" t="inlineStr">
+        <is>
+          <t>A close held for sign-off because verification recorded a variance</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>1. Attempt the sign-off as an operations user, a support user and a read-only finance user
+2. Attempt it as the Finance Lead</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>Every unauthorised attempt is rejected and audit-logged. Only the Finance Lead can seal a variance day, and the identity of the signer is stored on the close</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-22</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>A Rebuild Override Across an Unsealed Boundary Is Authorised and Recorded</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E23" s="28" t="inlineStr">
+        <is>
+          <t>A rebuild requested over a window containing an unsealed day</t>
+        </is>
+      </c>
+      <c r="F23" s="28" t="inlineStr">
+        <is>
+          <t>1. Attempt the override as an unauthorised user
+2. Perform it as the Finance Lead
+3. Inspect the rebuild run record</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="inlineStr">
+        <is>
+          <t>The unauthorised attempt is rejected. The authorised override succeeds and the run permanently records who overrode, when, and which unsealed boundary was crossed</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I23" s="29" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-23</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>Sealing and Unsealing Are Not Reachable by an Unauthorised Caller</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" s="28" t="inlineStr">
+        <is>
+          <t>API access to the daily close endpoints</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>1. Call the seal endpoint with a token lacking the finance privilege
+2. Attempt any unseal, update or delete route against a sealed close</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>The seal call is rejected at the API, not only hidden in the UI. No unseal, update or delete route exists or succeeds for any role, consistent with immutability</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I24" s="29" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Cutoff</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-24</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>The EOD Cutoff Honours the Configured Time Zone</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E25" s="28" t="inlineStr">
+        <is>
+          <t>Cutoff configured against a named business time zone; servers running in UTC</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>1. Post transactions either side of the configured local cutoff
+2. Run the close
+3. Inspect which business day each posting landed in</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>Day boundaries follow the configured business time zone, not the server clock. A posting just before local cutoff is in today; one just after is in tomorrow</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I25" s="29" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Cutoff</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-25</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>A Daylight-Saving Transition Produces Exactly One Close Per Wallet</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>A business time zone that observes a clock change; test dates covering both transitions</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>1. Run the close across the day the clock moves forward
+2. Run it across the day the clock moves back
+3. Count closes per wallet and check continuity</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>Exactly one sealed close per wallet per business day on both days. No day is skipped or duplicated, and continuity from the prior sealed closing still holds</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>Edge / Boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-26</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>A Day With No Postings Still Seals, With Opening Equal to Closing</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>A wallet with a sealed close for the prior day and no activity today</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>1. Run the close for the quiet day
+2. Inspect the record</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>A close is produced and sealed with zero day movement and closing identical to opening on every bucket. A quiet day is not skipped, because a gap would break the continuity chain and the rebuild anchor</t>
+        </is>
+      </c>
+      <c r="H27" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I27" s="29" t="inlineStr">
+        <is>
+          <t>Edge / Boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>Concurrency</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-27</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr">
+        <is>
+          <t>Two Concurrent EOD Runs Produce One Sealed Close</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>Ability to trigger the EOD job twice simultaneously</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>1. Trigger two EOD close runs for the same date and wallet at the same time
+2. Inspect the close records</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="inlineStr">
+        <is>
+          <t>Exactly one sealed close exists for that wallet and date. The second run is rejected or becomes a no-op; day movement is never counted twice</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I28" s="29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-28</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="inlineStr">
+        <is>
+          <t>Recorded Variance Is Carried on the Close Itself</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>A close sealed after Finance Lead sign-off on a recorded variance</t>
+        </is>
+      </c>
+      <c r="F29" s="28" t="inlineStr">
+        <is>
+          <t>1. Seal a variance day with sign-off
+2. Read the close record</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="inlineStr">
+        <is>
+          <t>The close carries the variance amount per bucket, the reason, the signer and the timestamp. The evidence is readable from the close without reconstructing it from job logs</t>
+        </is>
+      </c>
+      <c r="H29" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I29" s="29" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>TC-Close-29</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>Close Evidence Exports in Both CSV and PDF</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>Sealed closes for a date range</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>1. Export the range as CSV
+2. Export the same range as PDF
+3. Compare both against the sealed records</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="inlineStr">
+        <is>
+          <t>Both formats are produced and agree with the sealed records and with each other on every bucket. Amounts carry the platform monetary precision in SAR with no float rounding</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="I30" s="29" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I30"/>
   <conditionalFormatting sqref="H2:H21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Passed"</formula>

</xml_diff>